<commit_message>
Sizing: apply review corrections (incremental errors, queue-only hand-over cost, gated pessimistic ramp, cloud hosting, per-seat vendor price)
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -778,7 +778,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="170" fontId="34" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="15" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2023,14 +2023,14 @@
         </is>
       </c>
       <c r="C9" s="88" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="88" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="88" t="n">
+      <c r="E9" s="88" t="n">
         <v>8</v>
       </c>
-      <c r="E9" s="88" t="n">
-        <v>9</v>
-      </c>
       <c r="F9" s="84" t="inlineStr">
         <is>
           <t>analogy</t>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="G9" s="85" t="inlineStr">
         <is>
-          <t>Course order of magnitude: a human ticket costs EUR 5-15 all-in (S2 slides). Base 8 = agent time (row 10, ~5.2) x ~1.5 for team leads, QA and tools.</t>
+          <t>Course order of magnitude: a human ticket costs EUR 5-15 all-in (S2 slides). Base 7 = agent time (row 10, ~5.2) x ~1.35 for the part of team leads, QA and tools that scales with agent time.</t>
         </is>
       </c>
       <c r="H9" s="89" t="n"/>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="C39" s="94" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="D39" s="94" t="n">
         <v>0.15</v>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="G39" s="85" t="inlineStr">
         <is>
-          <t>Staged rollout: routing starts on low-critical tickets, each step conditional on a guardrail holding (template: staged like Octopus Energy).</t>
+          <t>Pessimistic = the guardrail fails and the rollout stops at about 10% (S4/Q1 gate), not a world with heavy errors and full ramp. Staged rollout: routing starts on low-critical tickets, each step conditional on a guardrail holding (template: staged like Octopus Energy).</t>
         </is>
       </c>
       <c r="H39" s="95" t="n"/>
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="C40" s="94" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="D40" s="94" t="n">
         <v>0.35</v>
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="C41" s="94" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="D41" s="94" t="n">
         <v>0.55</v>
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="C42" s="94" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D42" s="94" t="n">
         <v>0.7</v>
@@ -2862,7 +2862,7 @@
     <row r="45" ht="21.75" customHeight="1" s="68">
       <c r="A45" s="82" t="inlineStr">
         <is>
-          <t>AI cost per conversation (tokens, inference)</t>
+          <t>AI cost per time-saved-equivalent ticket (tokens, inference)</t>
         </is>
       </c>
       <c r="B45" s="82" t="inlineStr">
@@ -2946,13 +2946,13 @@
         </is>
       </c>
       <c r="C49" s="98" t="n">
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="D49" s="98" t="n">
-        <v>90000</v>
+        <v>80000</v>
       </c>
       <c r="E49" s="98" t="n">
-        <v>70000</v>
+        <v>60000</v>
       </c>
       <c r="F49" s="84" t="inlineStr">
         <is>
@@ -3006,13 +3006,13 @@
         </is>
       </c>
       <c r="C51" s="98" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="D51" s="98" t="n">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="E51" s="98" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="F51" s="84" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
     <row r="52" ht="15" customHeight="1" s="68">
       <c r="A52" s="82" t="inlineStr">
         <is>
-          <t>Supervision — humans in the loop (L2)</t>
+          <t>Quality owner - sampling audits, thresholds, upkeep</t>
         </is>
       </c>
       <c r="B52" s="82" t="inlineStr">
@@ -3038,13 +3038,13 @@
         </is>
       </c>
       <c r="C52" s="103" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="D52" s="103" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="E52" s="103" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="F52" s="84" t="inlineStr">
         <is>
@@ -3102,13 +3102,13 @@
         </is>
       </c>
       <c r="C54" s="98" t="n">
-        <v>40000</v>
+        <v>35000</v>
       </c>
       <c r="D54" s="98" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="E54" s="98" t="n">
-        <v>22000</v>
+        <v>18000</v>
       </c>
       <c r="F54" s="84" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="G54" s="85" t="inlineStr">
         <is>
-          <t>Monitoring, on-call and hosting of the self-hosted model endpoint (see Read options tab).</t>
+          <t>Monitoring, on-call and cloud hosting of the model endpoint (see Read options tab).</t>
         </is>
       </c>
       <c r="H54" s="99" t="n"/>
@@ -3166,10 +3166,10 @@
         </is>
       </c>
       <c r="C56" s="98" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="D56" s="98" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="E56" s="98" t="n">
         <v>3000</v>
@@ -3202,22 +3202,22 @@
         </is>
       </c>
       <c r="C59" s="94" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="D59" s="94" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="E59" s="94" t="n">
         <v>0.05</v>
       </c>
       <c r="F59" s="84" t="inlineStr">
         <is>
-          <t>guess</t>
+          <t>analogy</t>
         </is>
       </c>
       <c r="G59" s="85" t="inlineStr">
         <is>
-          <t>Agents get faster with experience and macros. Analogy: the course's do-nothing line for the class case (5%).</t>
+          <t>Agents get faster with experience and macros. The course class case uses 5% as the top of the range; base lower because our team has no stated tooling change.</t>
         </is>
       </c>
       <c r="H59" s="95" t="n"/>
@@ -3528,13 +3528,13 @@
         </is>
       </c>
       <c r="C7" s="115" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="D7" s="115" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="E7" s="115" t="n">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="F7" s="116" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
         <v>0.5</v>
       </c>
       <c r="D8" s="115" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="E8" s="115" t="n">
         <v>0.8</v>
@@ -3662,13 +3662,13 @@
         </is>
       </c>
       <c r="C12" s="115" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="D12" s="115" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="E12" s="115" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="F12" s="116" t="inlineStr">
         <is>
@@ -3799,13 +3799,13 @@
         </is>
       </c>
       <c r="C19" s="119" t="n">
-        <v>0.0015</v>
+        <v>0.001</v>
       </c>
       <c r="D19" s="119" t="n">
-        <v>0.001</v>
+        <v>0.0005</v>
       </c>
       <c r="E19" s="119" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0003</v>
       </c>
       <c r="F19" s="116" t="inlineStr">
         <is>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="G19" s="117" t="inlineStr">
         <is>
-          <t>Auto-route error that nobody catches, or wrong draft validated unread, with a real consequence. Test: seeded errors in S4 (hypothesis 4).</t>
+          <t>INCREMENTAL uncaught serious errors versus today (humans also misroute 1 in 7): auto-route error nobody catches, or wrong draft validated unread, with a real consequence. Test: seeded errors in S4 (hypothesis 4).</t>
         </is>
       </c>
     </row>
@@ -3830,13 +3830,13 @@
         </is>
       </c>
       <c r="C20" s="119" t="n">
-        <v>0.004</v>
+        <v>0.0025</v>
       </c>
       <c r="D20" s="119" t="n">
-        <v>0.0025</v>
+        <v>0.0012</v>
       </c>
       <c r="E20" s="119" t="n">
-        <v>0.0015</v>
+        <v>0.0007</v>
       </c>
       <c r="F20" s="116" t="inlineStr">
         <is>
@@ -3861,13 +3861,13 @@
         </is>
       </c>
       <c r="C21" s="119" t="n">
-        <v>0.0025</v>
+        <v>0.0015</v>
       </c>
       <c r="D21" s="119" t="n">
-        <v>0.0015</v>
+        <v>0.0008</v>
       </c>
       <c r="E21" s="119" t="n">
-        <v>0.001</v>
+        <v>0.0005</v>
       </c>
       <c r="F21" s="116" t="inlineStr">
         <is>
@@ -3919,13 +3919,13 @@
         </is>
       </c>
       <c r="C23" s="120" t="n">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
       <c r="D23" s="120" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="E23" s="120" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="F23" s="116" t="inlineStr">
         <is>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="G23" s="117" t="inlineStr">
         <is>
-          <t>Course order of magnitude EUR 0.02-0.20 per conversation. Recheck prices on the day.</t>
+          <t>About 5k tokens in and 500 out on a mid-size model; course order of magnitude EUR 0.02-0.20 per conversation. Recheck prices on the day.</t>
         </is>
       </c>
     </row>
@@ -4024,23 +4024,26 @@
           <t>share</t>
         </is>
       </c>
-      <c r="C27" s="115" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="D27" s="115" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E27" s="115" t="n">
-        <v>0.08</v>
+      <c r="C27" s="118">
+        <f>1-C13</f>
+        <v/>
+      </c>
+      <c r="D27" s="118">
+        <f>1-D13</f>
+        <v/>
+      </c>
+      <c r="E27" s="118">
+        <f>1-E13</f>
+        <v/>
       </c>
       <c r="F27" s="116" t="inlineStr">
         <is>
-          <t>guess</t>
+          <t>formula</t>
         </is>
       </c>
       <c r="G27" s="117" t="inlineStr">
         <is>
-          <t>Test: reroute counts in S4 (gold set) then S6.</t>
+          <t>Equal to 1 minus the correctly routed share of row 13. Test: reroute counts in S4 (gold set) then S6.</t>
         </is>
       </c>
     </row>
@@ -4056,14 +4059,14 @@
         </is>
       </c>
       <c r="C28" s="122" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="122" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="122" t="n">
         <v>4</v>
       </c>
-      <c r="D28" s="122" t="n">
-        <v>6</v>
-      </c>
-      <c r="E28" s="122" t="n">
-        <v>8</v>
-      </c>
       <c r="F28" s="116" t="inlineStr">
         <is>
           <t>guess</t>
@@ -4071,7 +4074,7 @@
       </c>
       <c r="G28" s="117" t="inlineStr">
         <is>
-          <t>About 5 min of two agents plus a queue delay. Test: time study.</t>
+          <t>Queue delay and merchant irritation only: the second desk re-reading is hands-on time already inside the 15% slice. Test: time study.</t>
         </is>
       </c>
     </row>
@@ -4189,14 +4192,14 @@
         </is>
       </c>
       <c r="C33" s="115" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D33" s="115" t="n">
         <v>0.7</v>
       </c>
-      <c r="D33" s="115" t="n">
+      <c r="E33" s="115" t="n">
         <v>0.8</v>
       </c>
-      <c r="E33" s="115" t="n">
-        <v>0.9</v>
-      </c>
       <c r="F33" s="116" t="inlineStr">
         <is>
           <t>guess</t>
@@ -4204,7 +4207,7 @@
       </c>
       <c r="G33" s="117" t="inlineStr">
         <is>
-          <t>A rule needs less ramp-up than a model.</t>
+          <t>A rule needs less ramp-up than a model, but it also has a build quarter.</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4406,7 @@
         </is>
       </c>
       <c r="C8" s="120" t="n">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -4428,7 +4431,7 @@
         </is>
       </c>
       <c r="C9" s="120" t="n">
-        <v>5</v>
+        <v>0.6</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -4482,7 +4485,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Self-hosted model endpoint, always on (small GPU)</t>
+          <t>Model endpoint in our cloud account - small fine-tuned model</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4491,7 +4494,7 @@
         </is>
       </c>
       <c r="C12" s="122" t="n">
-        <v>600</v>
+        <v>150</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -4500,7 +4503,7 @@
       </c>
       <c r="H12" s="112" t="inlineStr">
         <is>
-          <t>Cloud list price of a small GPU instance, 24/7. Could be lower with scale-to-zero or CPU for a very small model; the volume (1 ticket every 2 minutes) is low.</t>
+          <t>A small quantised model on a CPU VM or a serverless GPU that scales to zero (billed per second). A dedicated always-on GPU would be about EUR 600. Recheck the cloud price list.</t>
         </is>
       </c>
     </row>
@@ -4554,6 +4557,31 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Model endpoint - larger open-source model (7-30B), prompted only</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>EUR / month</t>
+        </is>
+      </c>
+      <c r="C15" s="122" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>guess</t>
+        </is>
+      </c>
+      <c r="H15" s="112" t="inlineStr">
+        <is>
+          <t>Needs a bigger GPU than the fine-tuned small model.</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
       <c r="A16" s="113" t="inlineStr">
         <is>
@@ -4649,11 +4677,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C - Open-source LLM, prompted, self-hosted</t>
+          <t>C - Open-source LLM, prompted, in our cloud account</t>
         </is>
       </c>
       <c r="C19" s="127">
-        <f>C12</f>
+        <f>C15</f>
         <v/>
       </c>
       <c r="D19" s="127">
@@ -4672,14 +4700,14 @@
       </c>
       <c r="H19" s="112" t="inlineStr">
         <is>
-          <t>Endpoint cost; a larger model may need a bigger GPU than D.</t>
+          <t>Larger model, bigger GPU than D.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>D - Small fine-tuned LLM, self-hosted</t>
+          <t>D - Small fine-tuned LLM, in our cloud account</t>
         </is>
       </c>
       <c r="C20" s="127">
@@ -4814,7 +4842,7 @@
     <row r="28">
       <c r="A28" s="130" t="inlineStr">
         <is>
-          <t>Reading: at this volume the external API is far cheaper than any self-hosted option, so cost alone cannot justify D. D (or C) is defended on data and control: tickets with payment data stay in-house, the model version is pinned, and there is no provider terms change or retirement. Whether that is worth the extra cost is a product decision for the Head of Compliance (memo). If S4 shows a prompted model is clearly less accurate or if the data constraint is dropped, we recommend E.</t>
+          <t>Reading: at this volume an external API is cheaper than any option in our cloud account, but the gap is a few thousand euros a year, small next to the value of accuracy (one point of routing accuracy is worth about EUR 14k a year in hand-overs). So choose D, C or E on accuracy on the gold set first; then on data and control (tickets with payment data stay in our tenancy, model version pinned, no provider retirement), a product decision for the Head of Compliance. The data argument only holds if the drafter, which sees more payment data than the router, is also kept in our tenancy or under an EU zero-retention contract.</t>
         </is>
       </c>
     </row>
@@ -6296,14 +6324,14 @@
     <row r="30" ht="15" customHeight="1" s="68">
       <c r="A30" s="131" t="inlineStr">
         <is>
-          <t>Base case, varying only the share of handling time saved on payment-status tickets (row 22 of Inputs). Everything else at Base; error and AI cost stay per ticket handled.</t>
+          <t>Base case, varying the total share of handling time saved (all categories). Everything else at Base; error and AI cost are per ticket handled, so they do not move.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="27.75" customHeight="1" s="68">
       <c r="A31" s="79" t="inlineStr">
         <is>
-          <t>Time saved on payment-status tickets</t>
+          <t>Total time saved (share of handling time)</t>
         </is>
       </c>
       <c r="B31" s="79" t="n"/>
@@ -6330,10 +6358,10 @@
     </row>
     <row r="32" ht="15" customHeight="1" s="68">
       <c r="A32" s="143" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="C32" s="135">
-        <f>((Upside!D9*Inputs!D34*12*Upside!D$5)*A32*Inputs!D$9-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D19*Inputs!D30-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D24*Inputs!D$46)+Upside!D25+Upside!D35-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
+        <f>Inputs!D6*12*Upside!D$5*A32*Inputs!D$9-Upside!D40-Upside!D41-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
         <v/>
       </c>
       <c r="D32" s="135">
@@ -6351,10 +6379,10 @@
     </row>
     <row r="33" ht="15" customHeight="1" s="68">
       <c r="A33" s="143" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="C33" s="135">
-        <f>((Upside!D9*Inputs!D34*12*Upside!D$5)*A33*Inputs!D$9-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D19*Inputs!D30-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D24*Inputs!D$46)+Upside!D25+Upside!D35-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
+        <f>Inputs!D6*12*Upside!D$5*A33*Inputs!D$9-Upside!D40-Upside!D41-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
         <v/>
       </c>
       <c r="D33" s="135">
@@ -6372,10 +6400,10 @@
     </row>
     <row r="34" ht="15" customHeight="1" s="68">
       <c r="A34" s="143" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="C34" s="135">
-        <f>((Upside!D9*Inputs!D34*12*Upside!D$5)*A34*Inputs!D$9-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D19*Inputs!D30-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D24*Inputs!D$46)+Upside!D25+Upside!D35-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
+        <f>Inputs!D6*12*Upside!D$5*A34*Inputs!D$9-Upside!D40-Upside!D41-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
         <v/>
       </c>
       <c r="D34" s="135">
@@ -6393,10 +6421,10 @@
     </row>
     <row r="35" ht="15" customHeight="1" s="68">
       <c r="A35" s="143" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="C35" s="135">
-        <f>((Upside!D9*Inputs!D34*12*Upside!D$5)*A35*Inputs!D$9-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D19*Inputs!D30-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D24*Inputs!D$46)+Upside!D25+Upside!D35-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
+        <f>Inputs!D6*12*Upside!D$5*A35*Inputs!D$9-Upside!D40-Upside!D41-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
         <v/>
       </c>
       <c r="D35" s="135">
@@ -6417,7 +6445,7 @@
         <v>0.3</v>
       </c>
       <c r="C36" s="135">
-        <f>((Upside!D9*Inputs!D34*12*Upside!D$5)*A36*Inputs!D$9-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D19*Inputs!D30-(Upside!D9*Inputs!D34*12*Upside!D$5)*Flow!D24*Inputs!D$46)+Upside!D25+Upside!D35-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
+        <f>Inputs!D6*12*Upside!D$5*A36*Inputs!D$9-Upside!D40-Upside!D41-D14+N(Inputs!$D$67)+N(Inputs!$D$68)</f>
         <v/>
       </c>
       <c r="D36" s="135">
@@ -6929,8 +6957,9 @@
         </is>
       </c>
       <c r="C22" s="144" t="n"/>
-      <c r="D22" s="155" t="n">
-        <v>0.9</v>
+      <c r="D22" s="155">
+        <f>25*45*12/Upside!D38</f>
+        <v/>
       </c>
       <c r="E22" s="156" t="inlineStr">
         <is>
@@ -6940,7 +6969,7 @@
       <c r="F22" s="144" t="n"/>
       <c r="G22" s="109" t="inlineStr">
         <is>
-          <t>guess from an analogy: Intercom Fin listed $0.99 per resolution in 2025 (template tip). A vendor copilot is more often priced per seat; here 'resolutions' are the time-saved-equivalent tickets of the Upside tab, so this is a rough proxy. Recheck.</t>
+          <t>Per-seat pricing expressed per time-saved-equivalent ticket: 25 seats x about EUR 45 a month (guess; vendor copilots are priced per seat; template tip: Intercom Fin listed $0.99 per resolution in 2025). Recheck the vendor price.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add data constraint, four-option comparison, staged-go positioning; sizing with private-cloud hosting
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -3102,13 +3102,13 @@
         </is>
       </c>
       <c r="C54" s="98" t="n">
-        <v>35000</v>
+        <v>70000</v>
       </c>
       <c r="D54" s="98" t="n">
-        <v>25000</v>
+        <v>45000</v>
       </c>
       <c r="E54" s="98" t="n">
-        <v>18000</v>
+        <v>30000</v>
       </c>
       <c r="F54" s="84" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="G54" s="85" t="inlineStr">
         <is>
-          <t>Monitoring, on-call and cloud hosting of the model endpoint (see Read options tab).</t>
+          <t>Monitoring and on-call (about 25k) plus hosting of two model endpoints in our own cloud: the router (small model) and the drafter (larger model, about EUR 1,500 a month). Data constraint: no external model API (README). See Read options tab.</t>
         </is>
       </c>
       <c r="H54" s="99" t="n"/>
@@ -3919,22 +3919,22 @@
         </is>
       </c>
       <c r="C23" s="120" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="D23" s="120" t="n">
-        <v>0.03</v>
+        <v>0.005</v>
       </c>
       <c r="E23" s="120" t="n">
-        <v>0.02</v>
+        <v>0.003</v>
       </c>
       <c r="F23" s="116" t="inlineStr">
         <is>
-          <t>analogy</t>
+          <t>guess</t>
         </is>
       </c>
       <c r="G23" s="117" t="inlineStr">
         <is>
-          <t>About 5k tokens in and 500 out on a mid-size model; course order of magnitude EUR 0.02-0.20 per conversation. Recheck prices on the day.</t>
+          <t>Self-hosted drafter: the marginal cost per ticket is near zero (retrieval, database queries, power); the endpoint is a fixed cost in Inputs row 54.</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4737,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E1 - External API, small model, prompted</t>
+          <t>E1 - External API, small model (REFERENCE ONLY, excluded)</t>
         </is>
       </c>
       <c r="C21" s="127">
@@ -4760,14 +4760,14 @@
       </c>
       <c r="H21" s="112" t="inlineStr">
         <is>
-          <t>tickets x (tokens in x price in + tokens out x price out).</t>
+          <t>Excluded by the data constraint: tickets never leave Keelpay's cloud. Shown to price the constraint.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E2 - External API, large model, prompted</t>
+          <t>E2 - External API, large model (REFERENCE ONLY, excluded)</t>
         </is>
       </c>
       <c r="C22" s="127">
@@ -4842,7 +4842,7 @@
     <row r="28">
       <c r="A28" s="130" t="inlineStr">
         <is>
-          <t>Reading: at this volume an external API is cheaper than any option in our cloud account, but the gap is a few thousand euros a year, small next to the value of accuracy (one point of routing accuracy is worth about EUR 14k a year in hand-overs). So choose D, C or E on accuracy on the gold set first; then on data and control (tickets with payment data stay in our tenancy, model version pinned, no provider retirement), a product decision for the Head of Compliance. The data argument only holds if the drafter, which sees more payment data than the router, is also kept in our tenancy or under an EU zero-retention contract.</t>
+          <t>Reading: the data constraint (README) removes E, so the real comparison is A, B, C and D inside our cloud. C is the true competitor of D: the drafter's larger model is already running, so prompting it to route adds almost no hosting. D therefore cannot be defended on hosting cost; it must win on the gold set (accuracy on urgent tickets, valid JSON, latency). E is shown only to price the constraint: running in our cloud costs a few thousand euros more a year than an external API, accepted because tickets carry merchant and payment data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sizing: scale-to-zero cloud hosting, growth in year-1 volume, steady-state reading
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -1930,10 +1930,10 @@
         <v>20000</v>
       </c>
       <c r="D6" s="83" t="n">
-        <v>20000</v>
+        <v>20500</v>
       </c>
       <c r="E6" s="83" t="n">
-        <v>20000</v>
+        <v>21000</v>
       </c>
       <c r="F6" s="84" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="G6" s="85" t="inlineStr">
         <is>
-          <t>Scenario data (README): ~20,000 tickets a month. Kept equal in the three scenarios.</t>
+          <t>Scenario data (README): ~20,000 tickets a month today. Base and High add the average year-1 effect of merchant growth (about +5% / +10% by year end); the do-nothing text in 01 says volume grows.</t>
         </is>
       </c>
       <c r="H6" s="86" t="n"/>
@@ -3102,13 +3102,13 @@
         </is>
       </c>
       <c r="C54" s="98" t="n">
-        <v>70000</v>
+        <v>40000</v>
       </c>
       <c r="D54" s="98" t="n">
-        <v>45000</v>
+        <v>20000</v>
       </c>
       <c r="E54" s="98" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="F54" s="84" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="G54" s="85" t="inlineStr">
         <is>
-          <t>Monitoring and on-call (about 25k) plus hosting of two model endpoints in our own cloud: the router (small model) and the drafter (larger model, about EUR 1,500 a month). Data constraint: no external model API (README). See Read options tab.</t>
+          <t>Mostly people time for monitoring and on-call. Hosting of the two endpoints in our own cloud (router and drafter, scale to zero, see Read options tab) is about EUR 2-3k a year. Data constraint: no external model API (README).</t>
         </is>
       </c>
       <c r="H54" s="99" t="n"/>
@@ -4485,7 +4485,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Model endpoint in our cloud account - small fine-tuned model</t>
+          <t>Router endpoint in our cloud account - small fine-tuned model, CPU, scale to zero</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4494,7 +4494,7 @@
         </is>
       </c>
       <c r="C12" s="122" t="n">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="H12" s="112" t="inlineStr">
         <is>
-          <t>A small quantised model on a CPU VM or a serverless GPU that scales to zero (billed per second). A dedicated always-on GPU would be about EUR 600. Recheck the cloud price list.</t>
+          <t>Container on Cloud Run with min-instances 0, billed per second, same pattern as the Museum Guide demo (free tier at its volume). 20,000 tickets x ~4 s x 2 vCPU is about 160k vCPU-seconds a month, around the free tier. Recheck the price list.</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4560,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Model endpoint - larger open-source model (7-30B), prompted only</t>
+          <t>Larger open-source model (7-30B), prompted - drafter class, GPU scale to zero</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4569,7 +4569,7 @@
         </is>
       </c>
       <c r="C15" s="122" t="n">
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -4578,7 +4578,7 @@
       </c>
       <c r="H15" s="112" t="inlineStr">
         <is>
-          <t>Needs a bigger GPU than the fine-tuned small model.</t>
+          <t>GPU billed per second, no always-on cost: tickets are processed asynchronously, so a cold start of tens of seconds is acceptable. About 20,000 x 15 s = 83 GPU-hours at roughly EUR 0.8-1 an hour. Recheck the price list.</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
     <row r="28">
       <c r="A28" s="130" t="inlineStr">
         <is>
-          <t>Reading: the data constraint (README) removes E, so the real comparison is A, B, C and D inside our cloud. C is the true competitor of D: the drafter's larger model is already running, so prompting it to route adds almost no hosting. D therefore cannot be defended on hosting cost; it must win on the gold set (accuracy on urgent tickets, valid JSON, latency). E is shown only to price the constraint: running in our cloud costs a few thousand euros more a year than an external API, accepted because tickets carry merchant and payment data.</t>
+          <t>Reading: the data constraint (README) removes E, so the real comparison is A, B, C and D inside our cloud. With scale-to-zero hosting (billed per second, as in the Museum Guide demo) all four cost tens of euros a month, far below the value of accuracy (one point of routing accuracy is worth about EUR 14k a year in hand-overs). So cost does not decide: D must win on the gold set (accuracy on urgent tickets, valid JSON, latency). E is shown only to price the constraint: a few tens of euros a month, so the constraint costs almost nothing and is cheap insurance for tickets that carry payment data.</t>
         </is>
       </c>
     </row>
@@ -5849,7 +5849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="54" customWidth="1" style="67" min="1" max="1"/>
@@ -6465,6 +6465,56 @@
       <c r="A38" s="131" t="inlineStr">
         <is>
           <t>Read down the table: the time-saved share at which the reading changes is the flip point. Name it in the memo - the S4 prototype and S6 A/B must measure it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="114" t="inlineStr">
+        <is>
+          <t>NOT IN THE TEMPLATE - additional readings used in the memo (the formula above stays as the course defines it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Base-case net annual value, year 1, above zero?</t>
+        </is>
+      </c>
+      <c r="D41">
+        <f>IF(D17&gt;0,"yes","no")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Expected value above zero and above the next-best project?</t>
+        </is>
+      </c>
+      <c r="D42">
+        <f>IF(AND(D19&gt;0,D19&gt;D23),"yes","no")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Base-case net value at steady-state adoption (Q4 level held for a full year)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EUR / yr</t>
+        </is>
+      </c>
+      <c r="D43" s="127">
+        <f>(Upside!D42+N(Inputs!D67))/Upside!D5*Inputs!D42-D14</f>
+        <v/>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Variable contribution and hand-overs scaled from the year-1 average ramp to the Q4 ramp, minus fixed costs. Year 1 carries the ramp-up; later years do not.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scale the scenario to 30,000 tickets a month; pessimistic case redefined as slow rollout
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -1927,13 +1927,13 @@
         </is>
       </c>
       <c r="C6" s="83" t="n">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="D6" s="83" t="n">
-        <v>20500</v>
+        <v>30750</v>
       </c>
       <c r="E6" s="83" t="n">
-        <v>21000</v>
+        <v>31500</v>
       </c>
       <c r="F6" s="84" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="G6" s="85" t="inlineStr">
         <is>
-          <t>Scenario data (README): ~20,000 tickets a month today. Base and High add the average year-1 effect of merchant growth (about +5% / +10% by year end); the do-nothing text in 01 says volume grows.</t>
+          <t>Scenario data (README): ~30,000 tickets a month today. Base and High add the average year-1 effect of merchant growth (about +5% / +10% by year end); the do-nothing text in 01 says volume grows.</t>
         </is>
       </c>
       <c r="H6" s="86" t="n"/>
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="C7" s="83" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="D7" s="83" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="E7" s="83" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="F7" s="84" t="inlineStr">
         <is>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="G7" s="85" t="inlineStr">
         <is>
-          <t>20,000 tickets x ~10 min hands-on / ~130 productive hours per agent. Test: headcount and timesheets of a real support team.</t>
+          <t>30,000 tickets x ~10 min hands-on / ~130 productive hours per agent. Test: headcount and timesheets of a real support team.</t>
         </is>
       </c>
       <c r="H7" s="86" t="n"/>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="C30" s="98" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="D30" s="98" t="n">
         <v>150</v>
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="C31" s="98" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="D31" s="98" t="n">
         <v>400</v>
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="C32" s="98" t="n">
-        <v>450</v>
+        <v>375</v>
       </c>
       <c r="D32" s="98" t="n">
         <v>300</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="C39" s="94" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="D39" s="94" t="n">
         <v>0.15</v>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="G39" s="85" t="inlineStr">
         <is>
-          <t>Pessimistic = the guardrail fails and the rollout stops at about 10% (S4/Q1 gate), not a world with heavy errors and full ramp. Staged rollout: routing starts on low-critical tickets, each step conditional on a guardrail holding (template: staged like Octopus Energy).</t>
+          <t>Pessimistic = a slow rollout, not a failed one: a failed rollout is stopped at the S4 gate (stage 2 is conditional). Staged rollout: routing starts on low-critical tickets, each step conditional on a guardrail holding (template: staged like Octopus Energy).</t>
         </is>
       </c>
       <c r="H39" s="95" t="n"/>
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="C40" s="94" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="D40" s="94" t="n">
         <v>0.35</v>
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="C41" s="94" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D41" s="94" t="n">
         <v>0.55</v>
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="C42" s="94" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D42" s="94" t="n">
         <v>0.7</v>
@@ -3799,7 +3799,7 @@
         </is>
       </c>
       <c r="C19" s="119" t="n">
-        <v>0.001</v>
+        <v>0.00075</v>
       </c>
       <c r="D19" s="119" t="n">
         <v>0.0005</v>
@@ -3830,7 +3830,7 @@
         </is>
       </c>
       <c r="C20" s="119" t="n">
-        <v>0.0025</v>
+        <v>0.0018</v>
       </c>
       <c r="D20" s="119" t="n">
         <v>0.0012</v>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="C21" s="119" t="n">
-        <v>0.0015</v>
+        <v>0.0012</v>
       </c>
       <c r="D21" s="119" t="n">
         <v>0.0008</v>

</xml_diff>

<commit_message>
Sizing: MVP-sized fixed costs; decision cell reads conditional go
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -2946,13 +2946,13 @@
         </is>
       </c>
       <c r="C49" s="98" t="n">
-        <v>110000</v>
+        <v>80000</v>
       </c>
       <c r="D49" s="98" t="n">
-        <v>80000</v>
+        <v>60000</v>
       </c>
       <c r="E49" s="98" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="F49" s="84" t="inlineStr">
         <is>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="G49" s="85" t="inlineStr">
         <is>
-          <t>Helpdesk and ledger integration, retrieval over desk policies, routing table, logging, review screen. Internal estimate; get a quote.</t>
+          <t>MVP integration: read-only helpdesk and ledger access, retrieval over desk policies, routing table, logging, review screen. About two engineers for three months at ~EUR 8-10k a month each. Internal estimate; get a quote.</t>
         </is>
       </c>
       <c r="H49" s="99" t="n"/>
@@ -3006,13 +3006,13 @@
         </is>
       </c>
       <c r="C51" s="98" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="D51" s="98" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E51" s="98" t="n">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="F51" s="84" t="inlineStr">
         <is>
@@ -3038,13 +3038,13 @@
         </is>
       </c>
       <c r="C52" s="103" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="D52" s="103" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E52" s="103" t="n">
-        <v>0.35</v>
+        <v>0.2</v>
       </c>
       <c r="F52" s="84" t="inlineStr">
         <is>
@@ -3102,13 +3102,13 @@
         </is>
       </c>
       <c r="C54" s="98" t="n">
-        <v>40000</v>
+        <v>18000</v>
       </c>
       <c r="D54" s="98" t="n">
-        <v>20000</v>
+        <v>12000</v>
       </c>
       <c r="E54" s="98" t="n">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="F54" s="84" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="G54" s="85" t="inlineStr">
         <is>
-          <t>Mostly people time for monitoring and on-call. Hosting of the two endpoints in our own cloud (router and drafter, scale to zero, see Read options tab) is about EUR 2-3k a year. Data constraint: no external model API (README).</t>
+          <t>Mostly people time for monitoring and on-call (the platform team already runs the helpdesk). Hosting of the two endpoints in our own cloud (router and drafter, scale to zero, see Read options tab) is about EUR 2-3k a year. Data constraint: no external model API (README).</t>
         </is>
       </c>
       <c r="H54" s="99" t="n"/>
@@ -3166,13 +3166,13 @@
         </is>
       </c>
       <c r="C56" s="98" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="D56" s="98" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="E56" s="98" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="F56" s="84" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rewrite investment memo and governance session 2 on the sizing; per-seat vendor price
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -4842,7 +4842,7 @@
     <row r="28">
       <c r="A28" s="130" t="inlineStr">
         <is>
-          <t>Reading: the data constraint (README) removes E, so the real comparison is A, B, C and D inside our cloud. With scale-to-zero hosting (billed per second, as in the Museum Guide demo) all four cost tens of euros a month, far below the value of accuracy (one point of routing accuracy is worth about EUR 14k a year in hand-overs). So cost does not decide: D must win on the gold set (accuracy on urgent tickets, valid JSON, latency). E is shown only to price the constraint: a few tens of euros a month, so the constraint costs almost nothing and is cheap insurance for tickets that carry payment data.</t>
+          <t>Reading: the data constraint (README) removes E, so the real comparison is A, B, C and D inside our cloud. With scale-to-zero hosting (billed per second, as in the Museum Guide demo) all four cost tens of euros a month, far below the value of accuracy (one point of routing accuracy is worth about EUR 11k a year in hand-overs). So cost does not decide: D must win on the gold set (accuracy on urgent tickets, valid JSON, latency). E is shown only to price the constraint: a few tens of euros a month, so the constraint costs almost nothing and is cheap insurance for tickets that carry payment data.</t>
         </is>
       </c>
     </row>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C22" s="144" t="n"/>
       <c r="D22" s="155">
-        <f>25*45*12/Upside!D38</f>
+        <f>Inputs!D7*45*12/Upside!D38</f>
         <v/>
       </c>
       <c r="E22" s="156" t="inlineStr">
@@ -7019,7 +7019,7 @@
       <c r="F22" s="144" t="n"/>
       <c r="G22" s="109" t="inlineStr">
         <is>
-          <t>Per-seat pricing expressed per time-saved-equivalent ticket: 25 seats x about EUR 45 a month (guess; vendor copilots are priced per seat; template tip: Intercom Fin listed $0.99 per resolution in 2025). Recheck the vendor price.</t>
+          <t>Per-seat pricing expressed per time-saved-equivalent ticket: one seat per support agent (Inputs row 7) x about EUR 45 a month (guess; vendor copilots are priced per seat; template tip: Intercom Fin listed $0.99 per resolution in 2025). Recheck the vendor price.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stale mentions after final review; add training and security review to integration cost
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -2038,7 +2038,7 @@
       </c>
       <c r="G9" s="85" t="inlineStr">
         <is>
-          <t>Course order of magnitude: a human ticket costs EUR 5-15 all-in (S2 slides). Base 7 = agent time (row 10, ~5.2) x ~1.35 for the part of team leads, QA and tools that scales with agent time.</t>
+          <t>Course order of magnitude: a human ticket costs EUR 5-15 all-in (S2 slides). Base 7 = agent time (row 10, ~5.15) x ~1.35 for the part of team leads, QA and tools that scales with agent time.</t>
         </is>
       </c>
       <c r="H9" s="89" t="n"/>
@@ -2946,13 +2946,13 @@
         </is>
       </c>
       <c r="C49" s="98" t="n">
-        <v>80000</v>
+        <v>105000</v>
       </c>
       <c r="D49" s="98" t="n">
-        <v>60000</v>
+        <v>85000</v>
       </c>
       <c r="E49" s="98" t="n">
-        <v>45000</v>
+        <v>65000</v>
       </c>
       <c r="F49" s="84" t="inlineStr">
         <is>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="G49" s="85" t="inlineStr">
         <is>
-          <t>MVP integration: read-only helpdesk and ledger access, retrieval over desk policies, routing table, logging, review screen. About two engineers for three months at ~EUR 8-10k a month each. Internal estimate; get a quote.</t>
+          <t>One-off: MVP integration (read-only helpdesk and ledger access, retrieval over desk policies, routing table, logging, review screen; about two engineers for three months, ~EUR 60k) plus training of the support agents, change management and the security and data-protection review (~EUR 25k). Internal estimate; get a quote.</t>
         </is>
       </c>
       <c r="H49" s="99" t="n"/>
@@ -4304,7 +4304,7 @@
     <row r="1">
       <c r="A1" s="111" t="inlineStr">
         <is>
-          <t>02_sizing - Read options: monthly cost of the five ways to read a ticket (step 1)</t>
+          <t>02_sizing - Read options: monthly cost of the ways to read a ticket (step 1)</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="H12" s="112" t="inlineStr">
         <is>
-          <t>Container on Cloud Run with min-instances 0, billed per second, same pattern as the Museum Guide demo (free tier at its volume). 20,000 tickets x ~4 s x 2 vCPU is about 160k vCPU-seconds a month, around the free tier. Recheck the price list.</t>
+          <t>Container on Cloud Run with min-instances 0, billed per second. 30,750 tickets x ~4 s x 2 vCPU is about 246k vCPU-seconds a month, a little above the free tier: a few euros. Same scale-to-zero pattern as the Museum Guide demo (CPU). Recheck the price list.</t>
         </is>
       </c>
     </row>
@@ -4578,7 +4578,7 @@
       </c>
       <c r="H15" s="112" t="inlineStr">
         <is>
-          <t>GPU billed per second, no always-on cost: tickets are processed asynchronously, so a cold start of tens of seconds is acceptable. About 20,000 x 15 s = 83 GPU-hours at roughly EUR 0.8-1 an hour. Recheck the price list.</t>
+          <t>GPU billed per second, no always-on cost: tickets are processed asynchronously, so a cold start of tens of seconds is acceptable. About 30,750 x 15 s = 128 GPU-hours at roughly EUR 0.8-1 an hour. The Museum Guide demo only shows CPU scale to zero; GPU cold starts of tens of seconds are assumed acceptable for asynchronous processing. Recheck the price list.</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
     <row r="28">
       <c r="A28" s="130" t="inlineStr">
         <is>
-          <t>Reading: the data constraint (README) removes E, so the real comparison is A, B, C and D inside our cloud. With scale-to-zero hosting (billed per second, as in the Museum Guide demo) all four cost tens of euros a month, far below the value of accuracy (one point of routing accuracy is worth about EUR 11k a year in hand-overs). So cost does not decide: D must win on the gold set (accuracy on urgent tickets, valid JSON, latency). E is shown only to price the constraint: a few tens of euros a month, so the constraint costs almost nothing and is cheap insurance for tickets that carry payment data.</t>
+          <t>Reading: the data constraint (README) removes E, so the real comparison is A, B, C and D inside our cloud. With scale-to-zero hosting (billed per second, as in the Museum Guide demo) all four cost tens of euros a month, far below the value of accuracy (one point of routing accuracy is worth about EUR 5k in year 1 (EUR 8k at steady state) from hand-overs alone). So cost does not decide: D must win on the gold set (accuracy on urgent tickets, valid JSON, latency). E is shown only to price the constraint: a few tens of euros a month, so the constraint costs almost nothing and is cheap insurance for tickets that carry payment data.</t>
         </is>
       </c>
     </row>
@@ -7019,7 +7019,7 @@
       <c r="F22" s="144" t="n"/>
       <c r="G22" s="109" t="inlineStr">
         <is>
-          <t>Per-seat pricing expressed per time-saved-equivalent ticket: one seat per support agent (Inputs row 7) x about EUR 45 a month (guess; vendor copilots are priced per seat; template tip: Intercom Fin listed $0.99 per resolution in 2025). Recheck the vendor price.</t>
+          <t>Per-seat pricing expressed per time-saved-equivalent ticket: one seat per support agent (Inputs row 7, 38) x about EUR 45 a month (guess; vendor copilots are priced per seat; template tip: Intercom Fin listed $0.99 per resolution in 2025). Recheck the vendor price.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Describe stage 1 as the transaction attach only
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -3252,7 +3252,7 @@
       </c>
       <c r="G60" s="85" t="inlineStr">
         <is>
-          <t>Next-best project: rules-only ticket-to-transaction attach plus routing on structured fields, no AI (value derived on the Flow tab). Name: 'rules-only attach'.</t>
+          <t>Next-best project: rules-only ticket-to-transaction attach, no AI (value derived on the Flow tab). Name: 'rules-only attach'.</t>
         </is>
       </c>
       <c r="H60" s="99" t="n"/>
@@ -4145,7 +4145,7 @@
     <row r="31">
       <c r="A31" s="114" t="inlineStr">
         <is>
-          <t>NEXT-BEST PROJECT - rules-only ticket-to-transaction attach and routing on structured fields (no AI)</t>
+          <t>NEXT-BEST PROJECT - rules-only ticket-to-transaction attach (no AI)</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="G32" s="117" t="inlineStr">
         <is>
-          <t>Removes the search for the payment (about half of slice B) for tickets with an ID or amount, and routes the structured part. Test: observe 20 tickets.</t>
+          <t>Removes the search for the payment (about half of slice B) for tickets with an ID or amount, Test: observe 20 tickets.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scale the case to 2,500 merchants and 36,000 tickets; port queue table and case card from the closed pitch PR
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -1927,13 +1927,13 @@
         </is>
       </c>
       <c r="C6" s="83" t="n">
-        <v>30000</v>
+        <v>36000</v>
       </c>
       <c r="D6" s="83" t="n">
-        <v>30750</v>
+        <v>36900</v>
       </c>
       <c r="E6" s="83" t="n">
-        <v>31500</v>
+        <v>37800</v>
       </c>
       <c r="F6" s="84" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="G6" s="85" t="inlineStr">
         <is>
-          <t>Scenario data (README): ~30,000 tickets a month today. Base and High add the average year-1 effect of merchant growth (about +5% / +10% by year end); the do-nothing text in 01 says volume grows.</t>
+          <t>Scenario data (README): ~36,000 tickets a month today. Base and High add the average year-1 effect of merchant growth (about +5% / +10% by year end); the do-nothing text in 01 says volume grows.</t>
         </is>
       </c>
       <c r="H6" s="86" t="n"/>
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="C7" s="83" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D7" s="83" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E7" s="83" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F7" s="84" t="inlineStr">
         <is>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="G7" s="85" t="inlineStr">
         <is>
-          <t>30,000 tickets x ~10 min hands-on / ~130 productive hours per agent. Test: headcount and timesheets of a real support team.</t>
+          <t>36,000 tickets x ~10 min hands-on / ~130 productive hours per agent. Test: headcount and timesheets of a real support team.</t>
         </is>
       </c>
       <c r="H7" s="86" t="n"/>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="H12" s="112" t="inlineStr">
         <is>
-          <t>Container on Cloud Run with min-instances 0, billed per second. 30,750 tickets x ~4 s x 2 vCPU is about 246k vCPU-seconds a month, a little above the free tier: a few euros. Same scale-to-zero pattern as the Museum Guide demo (CPU). Recheck the price list.</t>
+          <t>Container on Cloud Run with min-instances 0, billed per second. 36,900 tickets x ~4 s x 2 vCPU is about 295k vCPU-seconds a month, a little above the free tier: a few euros. Same scale-to-zero pattern as the Museum Guide demo (CPU). Recheck the price list.</t>
         </is>
       </c>
     </row>
@@ -4578,7 +4578,7 @@
       </c>
       <c r="H15" s="112" t="inlineStr">
         <is>
-          <t>GPU billed per second, no always-on cost: tickets are processed asynchronously, so a cold start of tens of seconds is acceptable. About 30,750 x 15 s = 128 GPU-hours at roughly EUR 0.8-1 an hour. The Museum Guide demo only shows CPU scale to zero; GPU cold starts of tens of seconds are assumed acceptable for asynchronous processing. Recheck the price list.</t>
+          <t>GPU billed per second, no always-on cost: tickets are processed asynchronously, so a cold start of tens of seconds is acceptable. About 36,900 x 15 s = 154 GPU-hours at roughly EUR 0.8-1 an hour. The Museum Guide demo only shows CPU scale to zero; GPU cold starts of tens of seconds are assumed acceptable for asynchronous processing. Recheck the price list.</t>
         </is>
       </c>
     </row>
@@ -7019,7 +7019,7 @@
       <c r="F22" s="144" t="n"/>
       <c r="G22" s="109" t="inlineStr">
         <is>
-          <t>Per-seat pricing expressed per time-saved-equivalent ticket: one seat per support agent (Inputs row 7, 38) x about EUR 45 a month (guess; vendor copilots are priced per seat; template tip: Intercom Fin listed $0.99 per resolution in 2025). Recheck the vendor price.</t>
+          <t>Per-seat pricing expressed per time-saved-equivalent ticket: one seat per support agent (Inputs row 7, 46) x about EUR 45 a month (guess; vendor copilots are priced per seat; template tip: Intercom Fin listed $0.99 per resolution in 2025). Recheck the vendor price.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sizing: in-between time-saved case (about 20 percent base); brief without minutes
</commit_message>
<xml_diff>
--- a/02_sizing.xlsx
+++ b/02_sizing.xlsx
@@ -3559,13 +3559,13 @@
         </is>
       </c>
       <c r="C8" s="115" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D8" s="115" t="n">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="E8" s="115" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="F8" s="116" t="inlineStr">
         <is>
@@ -3662,17 +3662,17 @@
         </is>
       </c>
       <c r="C12" s="115" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="D12" s="115" t="n">
-        <v>0.22</v>
+        <v>0.33</v>
       </c>
       <c r="E12" s="115" t="n">
-        <v>0.3</v>
+        <v>0.55</v>
       </c>
       <c r="F12" s="116" t="inlineStr">
         <is>
-          <t>analogy</t>
+          <t>guess</t>
         </is>
       </c>
       <c r="G12" s="117" t="inlineStr">

</xml_diff>